<commit_message>
Add 50-sample multitask workflow and update datasets
</commit_message>
<xml_diff>
--- a/Dataset/dataset_coverage.xlsx
+++ b/Dataset/dataset_coverage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/avijit/Desktop/IBM_LLM/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/avijit/Desktop/IndicJudge_IBM/Dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{889521F5-F32B-AD4C-BEB5-17F3F56BFFCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2F1B6DD-42F8-E54C-A0A9-42D2B9CF8A47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Coverage Matrix" sheetId="1" r:id="rId1"/>
@@ -222,23 +222,27 @@
       <b/>
       <sz val="12"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -302,11 +306,11 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -622,15 +626,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -987,7 +991,7 @@
       <c r="C17" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="D17" s="7" t="s">
         <v>38</v>
       </c>
       <c r="E17" s="4" t="s">

</xml_diff>